<commit_message>
Big update, removing most CBAM related stuff
</commit_message>
<xml_diff>
--- a/data/cost_data_init.xlsx
+++ b/data/cost_data_init.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terlouw_t\Documents\Projects\TRANSIENCE\P2_steel_db\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terlouw_t\Documents\Projects\TRANSIENCE\Steel_CBAM\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98BC97CA-727B-4BFB-AD60-45C0B65B244C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280C58A4-92F4-4847-B389-CF394063BF38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -246,9 +246,6 @@
     <t>land_m2_kw</t>
   </si>
   <si>
-    <t>ecoinvent_310_reference</t>
-  </si>
-  <si>
     <t>Electrolyzer (PEM)</t>
   </si>
   <si>
@@ -294,34 +291,37 @@
     <t>Here, we assume no hydrogen leakage during production to avoid double counting, since some of the LCIs include leakage already further up in the supply chain.</t>
   </si>
   <si>
-    <t>ecoinvent_image_SSP2-RCP26_2030_base</t>
-  </si>
-  <si>
-    <t>ecoinvent_image_SSP2-RCP26_2035_base</t>
-  </si>
-  <si>
-    <t>ecoinvent_image_SSP2-RCP26_2040_base</t>
-  </si>
-  <si>
-    <t>ecoinvent_image_SSP2-RCP26_2045_base</t>
-  </si>
-  <si>
-    <t>ecoinvent_image_SSP2-RCP26_2050_base</t>
-  </si>
-  <si>
-    <t>ecoinvent_remind_SSP2-PkBudg1150_2030_base</t>
-  </si>
-  <si>
-    <t>ecoinvent_remind_SSP2-PkBudg1150_2035_base</t>
-  </si>
-  <si>
-    <t>ecoinvent_remind_SSP2-PkBudg1150_2040_base</t>
-  </si>
-  <si>
-    <t>ecoinvent_remind_SSP2-PkBudg1150_2045_base</t>
-  </si>
-  <si>
-    <t>ecoinvent_remind_SSP2-PkBudg1150_2050_base</t>
+    <t>ecoinvent_remind_SSP2-PkBudg1000_2030_base</t>
+  </si>
+  <si>
+    <t>ecoinvent_remind_SSP2-PkBudg1000_2035_base</t>
+  </si>
+  <si>
+    <t>ecoinvent_remind_SSP2-PkBudg1000_2040_base</t>
+  </si>
+  <si>
+    <t>ecoinvent_remind_SSP2-PkBudg1000_2045_base</t>
+  </si>
+  <si>
+    <t>ecoinvent_remind_SSP2-PkBudg1000_2050_base</t>
+  </si>
+  <si>
+    <t>ecoinvent_image_SSP2-L_2030_base</t>
+  </si>
+  <si>
+    <t>ecoinvent_image_SSP2-L_2035_base</t>
+  </si>
+  <si>
+    <t>ecoinvent_image_SSP2-L_2040_base</t>
+  </si>
+  <si>
+    <t>ecoinvent_image_SSP2-L_2045_base</t>
+  </si>
+  <si>
+    <t>ecoinvent_image_SSP2-L_2050_base</t>
+  </si>
+  <si>
+    <t>ecoinvent_312_reference</t>
   </si>
 </sst>
 </file>
@@ -783,37 +783,37 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="J1" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="K1" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="L1" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="M1" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="M1" s="7" t="s">
-        <v>94</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>12</v>
@@ -3142,7 +3142,7 @@
     </row>
     <row r="45" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B45" t="s">
         <v>8</v>
@@ -3191,7 +3191,7 @@
         <v>8</v>
       </c>
       <c r="O45" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AB45">
         <v>2.5000000000000001E-2</v>
@@ -3229,7 +3229,7 @@
         <v>22</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C1" s="5">
         <v>2024</v>
@@ -3281,7 +3281,7 @@
         <v>euro/kW</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J2">
         <f>Sheet1!AB3</f>
@@ -3291,7 +3291,7 @@
     <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="10"/>
       <c r="B3" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C3" s="1">
         <f>Sheet1!C3</f>
@@ -3314,7 +3314,7 @@
         <v>-</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J3">
         <f>Sheet1!AB4</f>
@@ -3347,7 +3347,7 @@
         <v>years</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J4">
         <f>Sheet1!AB6</f>
@@ -3382,7 +3382,7 @@
         <v>euro/kW</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J5">
         <f>Sheet1!AB7</f>
@@ -3392,7 +3392,7 @@
     <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="10"/>
       <c r="B6" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C6" s="1">
         <f>Sheet1!C7</f>
@@ -3415,7 +3415,7 @@
         <v>-</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J6">
         <f>Sheet1!AB8</f>
@@ -3448,7 +3448,7 @@
         <v>years</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J7">
         <f>Sheet1!AB10</f>
@@ -3457,7 +3457,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>23</v>
@@ -3483,7 +3483,7 @@
         <v>euro/kW</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J8">
         <f>Sheet1!AB15</f>
@@ -3516,7 +3516,7 @@
         <v>-</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -3544,7 +3544,7 @@
         <v>years</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J10">
         <f>Sheet1!AB16</f>
@@ -3554,7 +3554,7 @@
     <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="11"/>
       <c r="B11" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C11" s="1">
         <f>Sheet1!C19</f>
@@ -3577,7 +3577,7 @@
         <v>-</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J11" t="e">
         <f>Sheet1!#REF!</f>
@@ -3611,13 +3611,13 @@
         <v>61</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="10"/>
       <c r="B13" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C13" s="1">
         <f>Sheet1!C21</f>
@@ -3640,7 +3640,7 @@
         <v>-</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -3669,7 +3669,7 @@
         <v>years</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -3698,7 +3698,7 @@
         <v>h</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -3727,7 +3727,7 @@
         <v>-</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -3756,7 +3756,7 @@
         <v>-</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -3785,7 +3785,7 @@
         <v>-</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -3814,7 +3814,7 @@
         <v>-</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -3843,7 +3843,7 @@
         <v>-</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -3872,12 +3872,12 @@
         <v>-</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>27</v>
@@ -3902,7 +3902,7 @@
         <v>8</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -3930,12 +3930,12 @@
         <v>14</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>27</v>
@@ -3960,7 +3960,7 @@
         <v>8</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -3988,7 +3988,7 @@
         <v>14</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.55000000000000004">

</xml_diff>